<commit_message>
Run Phase A4 Cohen's kappa on second annotator; fix reciprocity_hook taxonomy gap
Second annotator's 80-message subset imported to labels_second.jsonl.
Macro-kappa 0.68, above the plan's 0.6 threshold. Per-technique outlier:
reciprocity_hook kappa -0.02 (primary marked it 14/80, second only 1/80),
a genuine definitional gap rather than noise. counter_moves.yaml's own
source ("I4C advisory on lottery and prize-based frauds") already backed
the broader reading, so fixed by tightening RECIPROCITY_HOOK's wording in
taxonomy.py (feeds both the Layer 1 prompt and the labeling legend) rather
than relabeling data. The -0.02/0.68 numbers are kept as the honest
pre-fix evidence. Full writeup in ERROR_ANALYSIS.md.

Claude-Session: https://claude.ai/code/session_01UZM2TYFdT5QcGeNk7mLdtG
</commit_message>
<xml_diff>
--- a/backend/data/corpus/gold/gold_labeling_second.xlsx
+++ b/backend/data/corpus/gold/gold_labeling_second.xlsx
@@ -553,7 +553,11 @@
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="F2" s="3" t="inlineStr"/>
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="3" t="inlineStr"/>
@@ -562,7 +566,11 @@
       <c r="K2" s="3" t="inlineStr"/>
       <c r="L2" s="3" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
-      <c r="N2" s="3" t="inlineStr"/>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="O2" s="3" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
     </row>
@@ -582,7 +590,11 @@
           <t>Did u find a sitter for kaitlyn? I was sick and slept all day yesterday.</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr"/>
@@ -612,7 +624,11 @@
           <t>Yay can't wait to party together!</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="3" t="inlineStr"/>
       <c r="G4" s="3" t="inlineStr"/>
@@ -642,7 +658,11 @@
           <t>She said,'' do u mind if I go into the bedroom for a minute ? '' ''OK'', I sed in a sexy mood. She came out 5 minuts latr wid a cake...n My Wife,</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr"/>
@@ -672,7 +692,11 @@
           <t>Do you want a New Nokia 3510i colour phone DeliveredTomorrow? With 300 free minutes to any mobile + 100 free texts + Free Camcorder reply or call 08000930705</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3" t="inlineStr"/>
       <c r="G6" s="3" t="inlineStr"/>
@@ -702,7 +726,11 @@
           <t>"AH POOR BABY!HOPE URFEELING BETTERSN LUV! PROBTHAT OVERDOSE OF WORK HEY GO CAREFUL SPK 2 U SN LOTS OF LOVEJEN XXX."</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr"/>
       <c r="G7" s="3" t="inlineStr"/>
@@ -733,10 +761,22 @@
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I8" s="3" t="inlineStr"/>
       <c r="J8" s="3" t="inlineStr"/>
       <c r="K8" s="3" t="inlineStr"/>
@@ -762,7 +802,11 @@
           <t>Wen did you get so spiritual and deep. That's great</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="3" t="inlineStr"/>
@@ -792,7 +836,11 @@
           <t>Oi. Ami parchi na re. Kicchu kaaj korte iccha korche na. Phone ta tul na. Plz. Plz.</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3" t="inlineStr"/>
       <c r="G10" s="3" t="inlineStr"/>
@@ -822,7 +870,11 @@
           <t>I'll pick you up at about 5.15pm to go to taunton if you still want to come.</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr"/>
       <c r="G11" s="3" t="inlineStr"/>
@@ -854,10 +906,26 @@
       </c>
       <c r="D12" s="3" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J12" s="3" t="inlineStr"/>
       <c r="K12" s="3" t="inlineStr"/>
       <c r="L12" s="3" t="inlineStr"/>
@@ -882,7 +950,11 @@
           <t>Hi, it's Priya. Can you send me the notes from today's class when you get a chance? No rush, whenever you're free.</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr"/>
       <c r="G13" s="3" t="inlineStr"/>
@@ -913,14 +985,26 @@
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="F14" s="3" t="inlineStr"/>
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr"/>
       <c r="I14" s="3" t="inlineStr"/>
       <c r="J14" s="3" t="inlineStr"/>
-      <c r="K14" s="3" t="inlineStr"/>
-      <c r="L14" s="3" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="M14" s="3" t="inlineStr"/>
       <c r="N14" s="3" t="inlineStr"/>
       <c r="O14" s="3" t="inlineStr"/>
@@ -942,7 +1026,11 @@
           <t>We spend our days waiting for the ideal path to appear in front of us.. But what we forget is.. "paths are made by walking.. not by waiting.." Goodnight!</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr"/>
       <c r="G15" s="3" t="inlineStr"/>
@@ -972,7 +1060,11 @@
           <t>3 pa but not selected.</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="3" t="inlineStr"/>
       <c r="G16" s="3" t="inlineStr"/>
@@ -1002,7 +1094,11 @@
           <t>You are right. Meanwhile how's project twins comin up</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr"/>
       <c r="G17" s="3" t="inlineStr"/>
@@ -1032,7 +1128,11 @@
           <t>Kothi print out marandratha.</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="3" t="inlineStr"/>
       <c r="G18" s="3" t="inlineStr"/>
@@ -1063,17 +1163,29 @@
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="F19" s="3" t="inlineStr"/>
       <c r="G19" s="3" t="inlineStr"/>
       <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J19" s="3" t="inlineStr"/>
       <c r="K19" s="3" t="inlineStr"/>
       <c r="L19" s="3" t="inlineStr"/>
       <c r="M19" s="3" t="inlineStr"/>
       <c r="N19" s="3" t="inlineStr"/>
-      <c r="O19" s="3" t="inlineStr"/>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="P19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1092,7 +1204,11 @@
           <t xml:space="preserve">I thk ü gotta go home by urself. Cos i'll b going out shopping 4 my frens present. </t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="3" t="inlineStr"/>
       <c r="G20" s="3" t="inlineStr"/>
@@ -1122,7 +1238,11 @@
           <t>Want to send me a virtual hug?... I need one</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr"/>
       <c r="G21" s="3" t="inlineStr"/>
@@ -1153,12 +1273,20 @@
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="F22" s="3" t="inlineStr"/>
       <c r="G22" s="3" t="inlineStr"/>
       <c r="H22" s="3" t="inlineStr"/>
       <c r="I22" s="3" t="inlineStr"/>
-      <c r="J22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K22" s="3" t="inlineStr"/>
       <c r="L22" s="3" t="inlineStr"/>
       <c r="M22" s="3" t="inlineStr"/>
@@ -1182,7 +1310,11 @@
           <t>I‘m parked next to a MINI!!!! When are you coming in today do you think?</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr"/>
       <c r="G23" s="3" t="inlineStr"/>
@@ -1212,7 +1344,11 @@
           <t>*deep sigh* ... I miss you :-( ... I am really surprised you haven't gone to the net cafe yet to get to me ... Don't you miss me?</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="3" t="inlineStr"/>
       <c r="G24" s="3" t="inlineStr"/>
@@ -1243,14 +1379,26 @@
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="F25" s="3" t="inlineStr"/>
       <c r="G25" s="3" t="inlineStr"/>
       <c r="H25" s="3" t="inlineStr"/>
       <c r="I25" s="3" t="inlineStr"/>
       <c r="J25" s="3" t="inlineStr"/>
-      <c r="K25" s="3" t="inlineStr"/>
-      <c r="L25" s="3" t="inlineStr"/>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="M25" s="3" t="inlineStr"/>
       <c r="N25" s="3" t="inlineStr"/>
       <c r="O25" s="3" t="inlineStr"/>
@@ -1272,7 +1420,11 @@
           <t>Your free ringtone is waiting to be collected. Simply text the password "MIX" to 85069 to verify. Get Usher and Britney. FML, PO Box 5249, MK17 92H. 450Ppw 16</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="3" t="inlineStr"/>
       <c r="G26" s="3" t="inlineStr"/>
@@ -1302,7 +1454,11 @@
           <t>Ard 515 like dat. Y?</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3" t="inlineStr"/>
       <c r="G27" s="3" t="inlineStr"/>
@@ -1332,7 +1488,11 @@
           <t>Ugh its been a long day. I'm exhausted. Just want to cuddle up and take a nap</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E28" s="3" t="inlineStr"/>
       <c r="F28" s="3" t="inlineStr"/>
       <c r="G28" s="3" t="inlineStr"/>
@@ -1362,7 +1522,11 @@
           <t>Your OTP for the transaction of Rs 2,500 at Amazon is 483920. Valid for 10 minutes. Do not share this OTP with anyone.</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3" t="inlineStr"/>
       <c r="G29" s="3" t="inlineStr"/>
@@ -1392,7 +1556,11 @@
           <t>I didnt get anything da</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E30" s="3" t="inlineStr"/>
       <c r="F30" s="3" t="inlineStr"/>
       <c r="G30" s="3" t="inlineStr"/>
@@ -1422,7 +1590,11 @@
           <t>Wait.i will come out.. &amp;lt;#&amp;gt;  min:)</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3" t="inlineStr"/>
       <c r="G31" s="3" t="inlineStr"/>
@@ -1452,7 +1624,11 @@
           <t>Wat time ü wan today?</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E32" s="3" t="inlineStr"/>
       <c r="F32" s="3" t="inlineStr"/>
       <c r="G32" s="3" t="inlineStr"/>
@@ -1482,7 +1658,11 @@
           <t>Hmmm...k...but i want to change the field quickly da:-)i wanna get system administrator or network administrator..</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr"/>
       <c r="G33" s="3" t="inlineStr"/>
@@ -1512,7 +1692,11 @@
           <t>Update_Now - 12Mths Half Price Orange line rental: 400mins...Call MobileUpd8 on 08000839402 or call2optout=J5Q</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E34" s="3" t="inlineStr"/>
       <c r="F34" s="3" t="inlineStr"/>
       <c r="G34" s="3" t="inlineStr"/>
@@ -1542,7 +1726,11 @@
           <t>Please tell me you have some of that special stock you were talking about</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr"/>
       <c r="G35" s="3" t="inlineStr"/>
@@ -1572,7 +1760,11 @@
           <t>Almost there, see u in a sec</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="3" t="inlineStr"/>
       <c r="G36" s="3" t="inlineStr"/>
@@ -1603,7 +1795,11 @@
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="F37" s="3" t="inlineStr"/>
       <c r="G37" s="3" t="inlineStr"/>
       <c r="H37" s="3" t="inlineStr"/>
@@ -1632,7 +1828,11 @@
           <t>And he's apparently bffs with carly quick now</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr"/>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E38" s="3" t="inlineStr"/>
       <c r="F38" s="3" t="inlineStr"/>
       <c r="G38" s="3" t="inlineStr"/>
@@ -1662,7 +1862,11 @@
           <t>Sweet heart how are you?</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E39" s="3" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr"/>
       <c r="G39" s="3" t="inlineStr"/>
@@ -1693,15 +1897,27 @@
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr"/>
-      <c r="E40" s="3" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="F40" s="3" t="inlineStr"/>
       <c r="G40" s="3" t="inlineStr"/>
       <c r="H40" s="3" t="inlineStr"/>
       <c r="I40" s="3" t="inlineStr"/>
       <c r="J40" s="3" t="inlineStr"/>
-      <c r="K40" s="3" t="inlineStr"/>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L40" s="3" t="inlineStr"/>
-      <c r="M40" s="3" t="inlineStr"/>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="N40" s="3" t="inlineStr"/>
       <c r="O40" s="3" t="inlineStr"/>
       <c r="P40" s="2" t="inlineStr"/>
@@ -1722,7 +1938,11 @@
           <t>Sir, I need Velusamy sir's date of birth and company bank facilities details.</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E41" s="3" t="inlineStr"/>
       <c r="F41" s="3" t="inlineStr"/>
       <c r="G41" s="3" t="inlineStr"/>
@@ -1752,7 +1972,11 @@
           <t>I know where the  &amp;lt;#&amp;gt;  is, I'll be there around 5</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr"/>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E42" s="3" t="inlineStr"/>
       <c r="F42" s="3" t="inlineStr"/>
       <c r="G42" s="3" t="inlineStr"/>
@@ -1784,9 +2008,21 @@
       </c>
       <c r="D43" s="3" t="inlineStr"/>
       <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr"/>
-      <c r="G43" s="3" t="inlineStr"/>
-      <c r="H43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I43" s="3" t="inlineStr"/>
       <c r="J43" s="3" t="inlineStr"/>
       <c r="K43" s="3" t="inlineStr"/>
@@ -1812,7 +2048,11 @@
           <t>I think i am disturbing her da</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr"/>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E44" s="3" t="inlineStr"/>
       <c r="F44" s="3" t="inlineStr"/>
       <c r="G44" s="3" t="inlineStr"/>
@@ -1842,7 +2082,11 @@
           <t>Cashbin.co.uk (Get lots of cash this weekend!) www.cashbin.co.uk Dear Welcome to the weekend We have got our biggest and best EVER cash give away!! These..</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E45" s="3" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr"/>
       <c r="G45" s="3" t="inlineStr"/>
@@ -1872,7 +2116,11 @@
           <t>Orange brings you ringtones from all time Chart Heroes, with a free hit each week! Go to Ringtones &amp; Pics on wap. To stop receiving these tips reply STOP.</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E46" s="3" t="inlineStr"/>
       <c r="F46" s="3" t="inlineStr"/>
       <c r="G46" s="3" t="inlineStr"/>
@@ -1904,11 +2152,23 @@
       </c>
       <c r="D47" s="3" t="inlineStr"/>
       <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G47" s="3" t="inlineStr"/>
       <c r="H47" s="3" t="inlineStr"/>
-      <c r="I47" s="3" t="inlineStr"/>
-      <c r="J47" s="3" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K47" s="3" t="inlineStr"/>
       <c r="L47" s="3" t="inlineStr"/>
       <c r="M47" s="3" t="inlineStr"/>
@@ -1932,7 +2192,11 @@
           <t>Goodmorning sleeping ga.</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E48" s="3" t="inlineStr"/>
       <c r="F48" s="3" t="inlineStr"/>
       <c r="G48" s="3" t="inlineStr"/>
@@ -1962,7 +2226,11 @@
           <t>07732584351 - Rodger Burns - MSG = We tried to call you re your reply to our sms for a free nokia mobile + free camcorder. Please call now 08000930705 for delivery tomorrow</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E49" s="3" t="inlineStr"/>
       <c r="F49" s="3" t="inlineStr"/>
       <c r="G49" s="3" t="inlineStr"/>
@@ -1993,17 +2261,33 @@
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr"/>
-      <c r="E50" s="3" t="inlineStr"/>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="F50" s="3" t="inlineStr"/>
       <c r="G50" s="3" t="inlineStr"/>
-      <c r="H50" s="3" t="inlineStr"/>
-      <c r="I50" s="3" t="inlineStr"/>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J50" s="3" t="inlineStr"/>
       <c r="K50" s="3" t="inlineStr"/>
       <c r="L50" s="3" t="inlineStr"/>
       <c r="M50" s="3" t="inlineStr"/>
       <c r="N50" s="3" t="inlineStr"/>
-      <c r="O50" s="3" t="inlineStr"/>
+      <c r="O50" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="P50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
@@ -2022,7 +2306,11 @@
           <t>U can WIN £100 of Music Gift Vouchers every week starting NOW Txt the word DRAW to 87066 TsCs www.Idew.com SkillGame, 1Winaweek, age16. 150ppermessSubscription</t>
         </is>
       </c>
-      <c r="D51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E51" s="3" t="inlineStr"/>
       <c r="F51" s="3" t="inlineStr"/>
       <c r="G51" s="3" t="inlineStr"/>
@@ -2052,7 +2340,11 @@
           <t>Hey you can pay. With salary de. Only  &amp;lt;#&amp;gt; .</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr"/>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E52" s="3" t="inlineStr"/>
       <c r="F52" s="3" t="inlineStr"/>
       <c r="G52" s="3" t="inlineStr"/>
@@ -2082,7 +2374,11 @@
           <t>My sister got placed in birla soft da:-)</t>
         </is>
       </c>
-      <c r="D53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E53" s="3" t="inlineStr"/>
       <c r="F53" s="3" t="inlineStr"/>
       <c r="G53" s="3" t="inlineStr"/>
@@ -2112,7 +2408,11 @@
           <t>Oh shut it. Omg yesterday I had a dream that I had 2 kids both boys. I was so pissed. Not only about the kids but them being boys. I even told mark in my dream that he was changing diapers cause I'm not getting owed in the face.</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr"/>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E54" s="3" t="inlineStr"/>
       <c r="F54" s="3" t="inlineStr"/>
       <c r="G54" s="3" t="inlineStr"/>
@@ -2142,7 +2442,11 @@
           <t>She went to attend another two rounds today..but still did't reach home..</t>
         </is>
       </c>
-      <c r="D55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E55" s="3" t="inlineStr"/>
       <c r="F55" s="3" t="inlineStr"/>
       <c r="G55" s="3" t="inlineStr"/>
@@ -2174,10 +2478,22 @@
       </c>
       <c r="D56" s="3" t="inlineStr"/>
       <c r="E56" s="3" t="inlineStr"/>
-      <c r="F56" s="3" t="inlineStr"/>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G56" s="3" t="inlineStr"/>
-      <c r="H56" s="3" t="inlineStr"/>
-      <c r="I56" s="3" t="inlineStr"/>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J56" s="3" t="inlineStr"/>
       <c r="K56" s="3" t="inlineStr"/>
       <c r="L56" s="3" t="inlineStr"/>
@@ -2202,7 +2518,11 @@
           <t>Your PNR 4521789630 is confirmed. Train 12951, coach B4, seat 34. Boarding at Platform 3. Have a safe journey.</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr"/>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E57" s="3" t="inlineStr"/>
       <c r="F57" s="3" t="inlineStr"/>
       <c r="G57" s="3" t="inlineStr"/>
@@ -2232,7 +2552,11 @@
           <t>Are you the cutest girl in the world or what</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr"/>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E58" s="3" t="inlineStr"/>
       <c r="F58" s="3" t="inlineStr"/>
       <c r="G58" s="3" t="inlineStr"/>
@@ -2262,7 +2586,11 @@
           <t>Pls i wont belive god.not only jesus.</t>
         </is>
       </c>
-      <c r="D59" s="3" t="inlineStr"/>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E59" s="3" t="inlineStr"/>
       <c r="F59" s="3" t="inlineStr"/>
       <c r="G59" s="3" t="inlineStr"/>
@@ -2292,7 +2620,11 @@
           <t>Reply to win £100 weekly! What professional sport does Tiger Woods play? Send STOP to 87239 to end service</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr"/>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E60" s="3" t="inlineStr"/>
       <c r="F60" s="3" t="inlineStr"/>
       <c r="G60" s="3" t="inlineStr"/>
@@ -2324,11 +2656,23 @@
       </c>
       <c r="D61" s="3" t="inlineStr"/>
       <c r="E61" s="3" t="inlineStr"/>
-      <c r="F61" s="3" t="inlineStr"/>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G61" s="3" t="inlineStr"/>
       <c r="H61" s="3" t="inlineStr"/>
-      <c r="I61" s="3" t="inlineStr"/>
-      <c r="J61" s="3" t="inlineStr"/>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K61" s="3" t="inlineStr"/>
       <c r="L61" s="3" t="inlineStr"/>
       <c r="M61" s="3" t="inlineStr"/>
@@ -2352,7 +2696,11 @@
           <t>Ü still got lessons?  Ü in sch?</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr"/>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E62" s="3" t="inlineStr"/>
       <c r="F62" s="3" t="inlineStr"/>
       <c r="G62" s="3" t="inlineStr"/>
@@ -2382,7 +2730,11 @@
           <t>Will you come online today night</t>
         </is>
       </c>
-      <c r="D63" s="3" t="inlineStr"/>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E63" s="3" t="inlineStr"/>
       <c r="F63" s="3" t="inlineStr"/>
       <c r="G63" s="3" t="inlineStr"/>
@@ -2412,7 +2764,11 @@
           <t>Great. P diddy is my neighbor and comes for toothpaste every morning</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr"/>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E64" s="3" t="inlineStr"/>
       <c r="F64" s="3" t="inlineStr"/>
       <c r="G64" s="3" t="inlineStr"/>
@@ -2442,7 +2798,11 @@
           <t>It does it on its own. Most of the time it fixes my spelling. But sometimes it gets a completely diff word. Go figure</t>
         </is>
       </c>
-      <c r="D65" s="3" t="inlineStr"/>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E65" s="3" t="inlineStr"/>
       <c r="F65" s="3" t="inlineStr"/>
       <c r="G65" s="3" t="inlineStr"/>
@@ -2472,7 +2832,11 @@
           <t>I get out of class in bsn in like  &amp;lt;#&amp;gt;  minutes, you know where advising is?</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr"/>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E66" s="3" t="inlineStr"/>
       <c r="F66" s="3" t="inlineStr"/>
       <c r="G66" s="3" t="inlineStr"/>
@@ -2504,7 +2868,11 @@
       </c>
       <c r="D67" s="3" t="inlineStr"/>
       <c r="E67" s="3" t="inlineStr"/>
-      <c r="F67" s="3" t="inlineStr"/>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G67" s="3" t="inlineStr"/>
       <c r="H67" s="3" t="inlineStr"/>
       <c r="I67" s="3" t="inlineStr"/>
@@ -2532,7 +2900,11 @@
           <t>Honey ? Sweetheart ? Darling ? Sexy buns ? Sugar plum ? Loverboy ? I miss you, boytoy ... *smacks your ass* Did you go to the gym too ?</t>
         </is>
       </c>
-      <c r="D68" s="3" t="inlineStr"/>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E68" s="3" t="inlineStr"/>
       <c r="F68" s="3" t="inlineStr"/>
       <c r="G68" s="3" t="inlineStr"/>
@@ -2562,7 +2934,11 @@
           <t>Dear Customer, Rs 4,999.00 has been debited from your account ending 4521 on 02-Aug-26 towards UPI/DebitCard txn at Big Bazaar. Avl bal Rs 12,340.50.</t>
         </is>
       </c>
-      <c r="D69" s="3" t="inlineStr"/>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E69" s="3" t="inlineStr"/>
       <c r="F69" s="3" t="inlineStr"/>
       <c r="G69" s="3" t="inlineStr"/>
@@ -2592,7 +2968,11 @@
           <t>Bognor it is! Should be splendid at this time of year.</t>
         </is>
       </c>
-      <c r="D70" s="3" t="inlineStr"/>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E70" s="3" t="inlineStr"/>
       <c r="F70" s="3" t="inlineStr"/>
       <c r="G70" s="3" t="inlineStr"/>
@@ -2624,10 +3004,26 @@
       </c>
       <c r="D71" s="3" t="inlineStr"/>
       <c r="E71" s="3" t="inlineStr"/>
-      <c r="F71" s="3" t="inlineStr"/>
-      <c r="G71" s="3" t="inlineStr"/>
-      <c r="H71" s="3" t="inlineStr"/>
-      <c r="I71" s="3" t="inlineStr"/>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J71" s="3" t="inlineStr"/>
       <c r="K71" s="3" t="inlineStr"/>
       <c r="L71" s="3" t="inlineStr"/>
@@ -2652,7 +3048,11 @@
           <t>My friend, she's studying at warwick, we've planned to go shopping and to concert tmw, but it may be canceled, havn't seen  for ages, yeah we should get together sometime!</t>
         </is>
       </c>
-      <c r="D72" s="3" t="inlineStr"/>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E72" s="3" t="inlineStr"/>
       <c r="F72" s="3" t="inlineStr"/>
       <c r="G72" s="3" t="inlineStr"/>
@@ -2682,7 +3082,11 @@
           <t>Lol ok your forgiven :)</t>
         </is>
       </c>
-      <c r="D73" s="3" t="inlineStr"/>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E73" s="3" t="inlineStr"/>
       <c r="F73" s="3" t="inlineStr"/>
       <c r="G73" s="3" t="inlineStr"/>
@@ -2712,7 +3116,11 @@
           <t xml:space="preserve">Congrats! 1 year special cinema pass for 2 is yours. call 09061209465 now! C Suprman V, Matrix3, StarWars3, etc all 4 FREE! bx420-ip4-5we. 150pm. Dont miss out! </t>
         </is>
       </c>
-      <c r="D74" s="3" t="inlineStr"/>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E74" s="3" t="inlineStr"/>
       <c r="F74" s="3" t="inlineStr"/>
       <c r="G74" s="3" t="inlineStr"/>
@@ -2742,7 +3150,11 @@
           <t>You have won a guaranteed £200 award or even £1000 cashto claim UR award call free on 08000407165 (18+) 2 stop getstop on 88222 PHP</t>
         </is>
       </c>
-      <c r="D75" s="3" t="inlineStr"/>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E75" s="3" t="inlineStr"/>
       <c r="F75" s="3" t="inlineStr"/>
       <c r="G75" s="3" t="inlineStr"/>
@@ -2772,7 +3184,11 @@
           <t>Ü dun need to pick ur gf?</t>
         </is>
       </c>
-      <c r="D76" s="3" t="inlineStr"/>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E76" s="3" t="inlineStr"/>
       <c r="F76" s="3" t="inlineStr"/>
       <c r="G76" s="3" t="inlineStr"/>
@@ -2802,7 +3218,11 @@
           <t>Yeah just open chat and click friend lists. Then make the list. Easy as pie</t>
         </is>
       </c>
-      <c r="D77" s="3" t="inlineStr"/>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E77" s="3" t="inlineStr"/>
       <c r="F77" s="3" t="inlineStr"/>
       <c r="G77" s="3" t="inlineStr"/>
@@ -2832,7 +3252,11 @@
           <t>Your Swiggy order #4521 has been picked up and is on the way. Estimated delivery in 22 minutes. Track live at swiggy.com/track</t>
         </is>
       </c>
-      <c r="D78" s="3" t="inlineStr"/>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E78" s="3" t="inlineStr"/>
       <c r="F78" s="3" t="inlineStr"/>
       <c r="G78" s="3" t="inlineStr"/>
@@ -2862,7 +3286,11 @@
           <t>Change windows logoff sound..</t>
         </is>
       </c>
-      <c r="D79" s="3" t="inlineStr"/>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E79" s="3" t="inlineStr"/>
       <c r="F79" s="3" t="inlineStr"/>
       <c r="G79" s="3" t="inlineStr"/>
@@ -2892,7 +3320,11 @@
           <t>Noooooooo please. Last thing I need is stress. For once in your life be fair.</t>
         </is>
       </c>
-      <c r="D80" s="3" t="inlineStr"/>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E80" s="3" t="inlineStr"/>
       <c r="F80" s="3" t="inlineStr"/>
       <c r="G80" s="3" t="inlineStr"/>
@@ -2922,7 +3354,11 @@
           <t>FREE entry into our £250 weekly comp just send the word WIN to 80086 NOW. 18 T&amp;C www.txttowin.co.uk</t>
         </is>
       </c>
-      <c r="D81" s="3" t="inlineStr"/>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="E81" s="3" t="inlineStr"/>
       <c r="F81" s="3" t="inlineStr"/>
       <c r="G81" s="3" t="inlineStr"/>
@@ -2947,7 +3383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3070,7 +3506,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>An unsolicited gift, prize, or refund offer designed to create a felt obligation to respond.</t>
+          <t>An unsolicited gift, prize, or refund offer designed to create a felt obligation to respond — e.g. 'you've won a £2000 bonus, call to claim' counts on its own; the offer itself is the hook, no separate explicit request for a favor in return is needed.</t>
         </is>
       </c>
     </row>
@@ -3164,6 +3600,14 @@
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>reciprocity_hook: a bare prize-claim ('you've won, call to claim a £2000 bonus') counts on its own — you do NOT need an explicit 'do me a favor in return' ask for this to apply.</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>